<commit_message>
FEHLER bei HA und ev. HSD ERF
/100 überprüfen -> eventuell excel einstellung falsch (Zahl vs. Standard)

--Y Größenordnung HA stimmt nicht
</commit_message>
<xml_diff>
--- a/Lärmschadenstool_EXCEL/Lärmschadenstool.xlsx
+++ b/Lärmschadenstool_EXCEL/Lärmschadenstool.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dokumente_lokal\LÄRM Projekte\Quantifizierung von Lärmschadenskosten\GitHub Repository\Hessen_END_Healthiar\Lärmschadenstool_EXCEL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9429B309-3E10-4FDE-97A6-BA5C75FFA764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{189560E9-9AF9-4119-A3F6-E6C3572EA995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Frontend" sheetId="8" r:id="rId1"/>
-    <sheet name="Agglomeration road" sheetId="1" r:id="rId2"/>
-    <sheet name="Fragen" sheetId="11" r:id="rId3"/>
-    <sheet name="ERF HRA" sheetId="10" r:id="rId4"/>
-    <sheet name="5dB to 1dB refinement" sheetId="9" r:id="rId5"/>
-    <sheet name="Agglomeration rail" sheetId="2" r:id="rId6"/>
-    <sheet name="Agglomeration air" sheetId="3" r:id="rId7"/>
-    <sheet name="Agglomeration industry" sheetId="4" r:id="rId8"/>
-    <sheet name="Major roads " sheetId="5" r:id="rId9"/>
-    <sheet name="Major railways " sheetId="6" r:id="rId10"/>
-    <sheet name="Major airports" sheetId="7" r:id="rId11"/>
+    <sheet name="Hinweise" sheetId="12" r:id="rId1"/>
+    <sheet name="Frontend" sheetId="8" r:id="rId2"/>
+    <sheet name="Agglomeration road" sheetId="1" r:id="rId3"/>
+    <sheet name="Fragen" sheetId="11" r:id="rId4"/>
+    <sheet name="ERF HRA" sheetId="10" r:id="rId5"/>
+    <sheet name="5dB to 1dB refinement" sheetId="9" r:id="rId6"/>
+    <sheet name="Agglomeration rail" sheetId="2" r:id="rId7"/>
+    <sheet name="Agglomeration air" sheetId="3" r:id="rId8"/>
+    <sheet name="Agglomeration industry" sheetId="4" r:id="rId9"/>
+    <sheet name="Major roads " sheetId="5" r:id="rId10"/>
+    <sheet name="Major railways " sheetId="6" r:id="rId11"/>
+    <sheet name="Major airports" sheetId="7" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="150">
   <si>
     <t>L_den</t>
   </si>
@@ -556,6 +557,9 @@
   </si>
   <si>
     <t>in Annex 4: "All estimates are per person and per year" -&gt; also  Multiplikation mit Exponierten der Kategorie (zB Ballungsraum Straßen) notwendig</t>
+  </si>
+  <si>
+    <t>DALY pro 100.000</t>
   </si>
 </sst>
 </file>
@@ -754,7 +758,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -840,6 +844,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="4" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" xfId="5" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -848,12 +867,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -868,20 +881,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" xfId="5" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1353,6 +1363,45 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11457340-40AB-4C39-9488-F3F169CC7A0E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D15C0212-0B91-4E6B-BA83-4D03E3220F57}">
+  <sheetPr codeName="Tabelle5"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D784C34-E246-472E-88D5-CA0D5063A3C9}">
+  <sheetPr codeName="Tabelle6"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70D71C91-7A22-40CF-B195-068A9D60F08B}">
+  <sheetPr codeName="Tabelle7"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C7D27E-13C9-40A4-936B-06BBF9BE4E35}">
   <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1380,15 +1429,15 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="74.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="51"/>
-      <c r="C5" s="51"/>
-      <c r="D5" s="51"/>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
-      <c r="G5" s="51"/>
+      <c r="B5" s="60"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
     </row>
     <row r="8" spans="1:15" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
@@ -1397,29 +1446,29 @@
     </row>
     <row r="9" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:15" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="52" t="s">
+      <c r="A10" s="61" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="52"/>
+      <c r="B10" s="61"/>
     </row>
     <row r="11" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C12" s="53" t="s">
+      <c r="C12" s="62" t="s">
         <v>73</v>
       </c>
-      <c r="D12" s="53"/>
-      <c r="E12" s="53"/>
-      <c r="F12" s="53"/>
-      <c r="G12" s="53"/>
-      <c r="H12" s="53"/>
-      <c r="J12" s="53" t="s">
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
+      <c r="G12" s="62"/>
+      <c r="H12" s="62"/>
+      <c r="J12" s="62" t="s">
         <v>74</v>
       </c>
-      <c r="K12" s="53"/>
-      <c r="L12" s="53"/>
-      <c r="M12" s="53"/>
-      <c r="N12" s="53"/>
-      <c r="O12" s="53"/>
+      <c r="K12" s="62"/>
+      <c r="L12" s="62"/>
+      <c r="M12" s="62"/>
+      <c r="N12" s="62"/>
+      <c r="O12" s="62"/>
     </row>
     <row r="13" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="C13" s="1" t="s">
@@ -1460,7 +1509,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="54" t="s">
+      <c r="A14" s="63" t="s">
         <v>49</v>
       </c>
       <c r="B14" t="s">
@@ -1507,7 +1556,7 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="54"/>
+      <c r="A15" s="63"/>
       <c r="B15" t="s">
         <v>84</v>
       </c>
@@ -1582,7 +1631,7 @@
       <c r="O17" s="8"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="54" t="s">
+      <c r="A18" s="63" t="s">
         <v>78</v>
       </c>
       <c r="B18" t="s">
@@ -1629,7 +1678,7 @@
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="54"/>
+      <c r="A19" s="63"/>
       <c r="B19" t="s">
         <v>80</v>
       </c>
@@ -1704,7 +1753,7 @@
       <c r="O21" s="8"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="54" t="s">
+      <c r="A22" s="63" t="s">
         <v>81</v>
       </c>
       <c r="B22" t="s">
@@ -1751,7 +1800,7 @@
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="54"/>
+      <c r="A23" s="63"/>
       <c r="B23" t="s">
         <v>83</v>
       </c>
@@ -1802,10 +1851,10 @@
     </row>
     <row r="31" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:15" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="52" t="s">
+      <c r="A32" s="61" t="s">
         <v>142</v>
       </c>
-      <c r="B32" s="52"/>
+      <c r="B32" s="61"/>
     </row>
     <row r="33" spans="2:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
@@ -1858,11 +1907,11 @@
       <c r="B39" s="44" t="s">
         <v>105</v>
       </c>
-      <c r="C39" s="66">
+      <c r="C39" s="56">
         <f>'Agglomeration road'!C82</f>
         <v>439746126.72747183</v>
       </c>
-      <c r="D39" s="66">
+      <c r="D39" s="56">
         <f>'Agglomeration road'!D82</f>
         <v>19474523816.498829</v>
       </c>
@@ -1883,30 +1932,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D784C34-E246-472E-88D5-CA0D5063A3C9}">
-  <sheetPr codeName="Tabelle6"/>
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70D71C91-7A22-40CF-B195-068A9D60F08B}">
-  <sheetPr codeName="Tabelle7"/>
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:U82"/>
+  <dimension ref="A1:U84"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" customWidth="1"/>
@@ -2416,21 +2445,21 @@
     <row r="39" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C40" s="15"/>
-      <c r="D40" s="57" t="s">
+      <c r="D40" s="64" t="s">
         <v>92</v>
       </c>
-      <c r="E40" s="57"/>
-      <c r="F40" s="57"/>
-      <c r="G40" s="57"/>
-      <c r="H40" s="57"/>
-      <c r="I40" s="57"/>
-      <c r="J40" s="57" t="s">
+      <c r="E40" s="64"/>
+      <c r="F40" s="64"/>
+      <c r="G40" s="64"/>
+      <c r="H40" s="64"/>
+      <c r="I40" s="64"/>
+      <c r="J40" s="64" t="s">
         <v>91</v>
       </c>
-      <c r="K40" s="57"/>
-      <c r="L40" s="57"/>
-      <c r="M40" s="57"/>
-      <c r="N40" s="57"/>
+      <c r="K40" s="64"/>
+      <c r="L40" s="64"/>
+      <c r="M40" s="64"/>
+      <c r="N40" s="64"/>
     </row>
     <row r="41" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="D41" s="15" t="s">
@@ -2471,10 +2500,10 @@
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A42" s="58" t="s">
+      <c r="A42" s="65" t="s">
         <v>102</v>
       </c>
-      <c r="B42" s="64" t="s">
+      <c r="B42" s="54" t="s">
         <v>85</v>
       </c>
       <c r="C42" s="20"/>
@@ -2533,7 +2562,7 @@
       <c r="U42" s="8"/>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A43" s="60"/>
+      <c r="A43" s="67"/>
       <c r="B43" s="15" t="s">
         <v>108</v>
       </c>
@@ -2574,7 +2603,7 @@
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A44" s="59"/>
+      <c r="A44" s="66"/>
       <c r="B44" s="24" t="s">
         <v>109</v>
       </c>
@@ -2637,7 +2666,7 @@
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A46" s="58" t="s">
+      <c r="A46" s="65" t="s">
         <v>57</v>
       </c>
       <c r="B46" s="19" t="s">
@@ -2691,7 +2720,7 @@
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A47" s="60"/>
+      <c r="A47" s="67"/>
       <c r="B47" s="15" t="s">
         <v>89</v>
       </c>
@@ -2749,7 +2778,7 @@
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A48" s="60"/>
+      <c r="A48" s="67"/>
       <c r="B48" s="15" t="s">
         <v>111</v>
       </c>
@@ -2774,8 +2803,8 @@
       <c r="O48" s="15"/>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A49" s="59"/>
-      <c r="B49" s="63" t="s">
+      <c r="A49" s="66"/>
+      <c r="B49" s="53" t="s">
         <v>135</v>
       </c>
       <c r="C49" s="43">
@@ -2799,7 +2828,7 @@
       <c r="O49" s="18"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A50" s="58" t="s">
+      <c r="A50" s="65" t="s">
         <v>62</v>
       </c>
       <c r="B50" s="19" t="s">
@@ -2853,7 +2882,7 @@
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A51" s="60"/>
+      <c r="A51" s="67"/>
       <c r="B51" s="15" t="s">
         <v>89</v>
       </c>
@@ -2911,7 +2940,7 @@
       </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A52" s="60"/>
+      <c r="A52" s="67"/>
       <c r="B52" s="15" t="s">
         <v>111</v>
       </c>
@@ -2936,8 +2965,8 @@
       <c r="O52" s="15"/>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A53" s="59"/>
-      <c r="B53" s="63" t="s">
+      <c r="A53" s="66"/>
+      <c r="B53" s="53" t="s">
         <v>136</v>
       </c>
       <c r="C53" s="43">
@@ -2961,7 +2990,7 @@
       <c r="O53" s="18"/>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A54" s="58" t="s">
+      <c r="A54" s="65" t="s">
         <v>65</v>
       </c>
       <c r="B54" s="19" t="s">
@@ -3015,7 +3044,7 @@
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A55" s="60"/>
+      <c r="A55" s="67"/>
       <c r="B55" s="15" t="s">
         <v>89</v>
       </c>
@@ -3073,7 +3102,7 @@
       </c>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A56" s="60"/>
+      <c r="A56" s="67"/>
       <c r="B56" s="15" t="s">
         <v>111</v>
       </c>
@@ -3098,8 +3127,8 @@
       <c r="O56" s="15"/>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A57" s="59"/>
-      <c r="B57" s="63" t="s">
+      <c r="A57" s="66"/>
+      <c r="B57" s="53" t="s">
         <v>137</v>
       </c>
       <c r="C57" s="43">
@@ -3123,7 +3152,7 @@
       <c r="O57" s="18"/>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A58" s="58" t="s">
+      <c r="A58" s="65" t="s">
         <v>69</v>
       </c>
       <c r="B58" s="19" t="s">
@@ -3177,7 +3206,7 @@
       </c>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A59" s="60"/>
+      <c r="A59" s="67"/>
       <c r="B59" s="15" t="s">
         <v>89</v>
       </c>
@@ -3235,7 +3264,7 @@
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A60" s="60"/>
+      <c r="A60" s="67"/>
       <c r="B60" s="15" t="s">
         <v>111</v>
       </c>
@@ -3260,8 +3289,8 @@
       <c r="O60" s="15"/>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A61" s="59"/>
-      <c r="B61" s="63" t="s">
+      <c r="A61" s="66"/>
+      <c r="B61" s="53" t="s">
         <v>138</v>
       </c>
       <c r="C61" s="22">
@@ -3285,7 +3314,7 @@
       <c r="O61" s="18"/>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A62" s="58" t="s">
+      <c r="A62" s="68" t="s">
         <v>45</v>
       </c>
       <c r="B62" s="34" t="s">
@@ -3337,7 +3366,7 @@
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A63" s="54"/>
+      <c r="A63" s="69"/>
       <c r="B63" s="34" t="s">
         <v>112</v>
       </c>
@@ -3387,7 +3416,7 @@
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A64" s="54"/>
+      <c r="A64" s="69"/>
       <c r="B64" s="15" t="s">
         <v>111</v>
       </c>
@@ -3402,8 +3431,8 @@
       <c r="E64" s="23"/>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A65" s="59"/>
-      <c r="B65" s="65" t="s">
+      <c r="A65" s="70"/>
+      <c r="B65" s="55" t="s">
         <v>139</v>
       </c>
       <c r="C65" s="36">
@@ -3503,7 +3532,7 @@
       <c r="O68" s="15"/>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A69" s="58" t="s">
+      <c r="A69" s="65" t="s">
         <v>102</v>
       </c>
       <c r="B69" s="20" t="s">
@@ -3557,7 +3586,7 @@
       <c r="O69" s="15"/>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A70" s="60"/>
+      <c r="A70" s="67"/>
       <c r="B70" s="15" t="s">
         <v>108</v>
       </c>
@@ -3596,7 +3625,7 @@
       <c r="O70" s="15"/>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A71" s="59"/>
+      <c r="A71" s="66"/>
       <c r="B71" s="24" t="s">
         <v>109</v>
       </c>
@@ -3668,7 +3697,7 @@
       <c r="O72" s="15"/>
     </row>
     <row r="73" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="55" t="s">
+      <c r="A73" s="71" t="s">
         <v>53</v>
       </c>
       <c r="B73" s="34" t="s">
@@ -3716,7 +3745,7 @@
       </c>
     </row>
     <row r="74" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="55"/>
+      <c r="A74" s="71"/>
       <c r="B74" s="34" t="s">
         <v>112</v>
       </c>
@@ -3762,7 +3791,7 @@
       </c>
     </row>
     <row r="75" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="55"/>
+      <c r="A75" s="71"/>
       <c r="B75" s="15" t="s">
         <v>111</v>
       </c>
@@ -3776,8 +3805,8 @@
       </c>
     </row>
     <row r="76" spans="1:15" s="34" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="56"/>
-      <c r="B76" s="65" t="s">
+      <c r="A76" s="70"/>
+      <c r="B76" s="55" t="s">
         <v>139</v>
       </c>
       <c r="C76" s="36">
@@ -3823,11 +3852,11 @@
       <c r="B81" s="44" t="s">
         <v>99</v>
       </c>
-      <c r="C81" s="61">
+      <c r="C81" s="51">
         <f>C61+C65+C76</f>
         <v>6282.0875246781688</v>
       </c>
-      <c r="D81" s="61">
+      <c r="D81" s="51">
         <f>D49+D53+D57+D65+D76</f>
         <v>278207.48309284041</v>
       </c>
@@ -3840,11 +3869,11 @@
       <c r="B82" s="44" t="s">
         <v>105</v>
       </c>
-      <c r="C82" s="62">
+      <c r="C82" s="52">
         <f>C81*70000</f>
         <v>439746126.72747183</v>
       </c>
-      <c r="D82" s="62">
+      <c r="D82" s="52">
         <f>D81*70000</f>
         <v>19474523816.498829</v>
       </c>
@@ -3854,6 +3883,11 @@
       </c>
       <c r="F82" t="s">
         <v>132</v>
+      </c>
+    </row>
+    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B84" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -3874,7 +3908,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B1B57BF-B5FC-49D0-8C1C-84AA1C3FC65A}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3898,7 +3932,7 @@
       <c r="A2" s="47">
         <v>1</v>
       </c>
-      <c r="B2" s="67" t="s">
+      <c r="B2" s="57" t="s">
         <v>109</v>
       </c>
       <c r="C2" s="49" t="s">
@@ -3909,7 +3943,7 @@
       <c r="A3" s="47">
         <v>2</v>
       </c>
-      <c r="B3" s="68" t="s">
+      <c r="B3" s="58" t="s">
         <v>107</v>
       </c>
       <c r="C3" s="48" t="s">
@@ -3920,7 +3954,7 @@
       <c r="A4" s="47">
         <v>3</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="59" t="s">
         <v>145</v>
       </c>
       <c r="C4" s="48" t="s">
@@ -3931,7 +3965,7 @@
       <c r="A5" s="47">
         <v>4</v>
       </c>
-      <c r="B5" s="68" t="s">
+      <c r="B5" s="58" t="s">
         <v>133</v>
       </c>
       <c r="C5" t="s">
@@ -3942,7 +3976,7 @@
       <c r="A6" s="50">
         <v>5</v>
       </c>
-      <c r="B6" s="68" t="s">
+      <c r="B6" s="58" t="s">
         <v>134</v>
       </c>
       <c r="C6" t="s">
@@ -3954,7 +3988,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46A8C717-7812-4473-9D8B-3495A5B0BB7F}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3964,7 +3998,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3AA0BE1-EB71-4657-B503-300F880C587F}">
   <dimension ref="A2:A3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3987,7 +4021,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC3BA502-77FB-4AA9-A654-F467290EB112}">
   <sheetPr codeName="Tabelle2"/>
   <dimension ref="A1:G13"/>
@@ -4176,7 +4210,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{601D2B11-F41E-4CFB-A90C-BC8CA1A15B8D}">
   <sheetPr codeName="Tabelle3"/>
   <dimension ref="A1"/>
@@ -4186,7 +4220,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B738CEAF-BA8D-46A4-B41F-A105DC1BD636}">
   <sheetPr codeName="Tabelle4"/>
   <dimension ref="A1"/>
@@ -4194,14 +4228,4 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D15C0212-0B91-4E6B-BA83-4D03E3220F57}">
-  <sheetPr codeName="Tabelle5"/>
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>